<commit_message>
pre-submission to Opt. Express
</commit_message>
<xml_diff>
--- a/AsymReca_ThkCalc.xlsb.xlsx
+++ b/AsymReca_ThkCalc.xlsb.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2024-ILLUSTRIOUS\My Drive (61050734@kmitl.ac.th)\AsymReca_SbSe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16E114B4-4BB6-4FF3-8C5E-C573438A4DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1669333-4FB3-455D-9BDB-86864CBD6862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532_back" sheetId="15" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="181">
   <si>
     <t>Wavelength (nm)</t>
   </si>
@@ -2169,6 +2169,15 @@
   </si>
   <si>
     <t>(SbSe/MgF/SbSe)^7</t>
+  </si>
+  <si>
+    <t>Si_amo_20°</t>
+  </si>
+  <si>
+    <t>0..000092</t>
+  </si>
+  <si>
+    <t>λ = 740</t>
   </si>
 </sst>
 </file>
@@ -2987,51 +2996,51 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3056,15 +3065,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -3074,6 +3083,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -3083,8 +3095,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3096,30 +3129,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3621,10 +3630,10 @@
       <c r="A1" s="147" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="149" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
       <c r="D1" s="44" t="s">
@@ -3636,27 +3645,27 @@
       <c r="F1" s="155" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="162" t="s">
+      <c r="G1" s="157" t="s">
         <v>116</v>
       </c>
       <c r="H1" s="159" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="151" t="s">
+      <c r="I1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="153"/>
-      <c r="K1" s="161"/>
-      <c r="L1" s="151" t="s">
+      <c r="K1" s="162"/>
+      <c r="L1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="M1" s="153"/>
-      <c r="N1" s="161"/>
-      <c r="O1" s="151" t="s">
+      <c r="N1" s="162"/>
+      <c r="O1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="P1" s="153"/>
-      <c r="Q1" s="161"/>
+      <c r="Q1" s="162"/>
       <c r="S1" s="128"/>
       <c r="T1" s="128"/>
       <c r="U1" s="128"/>
@@ -3664,12 +3673,12 @@
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="152"/>
       <c r="D2" s="44"/>
       <c r="E2" s="154"/>
       <c r="F2" s="156"/>
-      <c r="G2" s="163"/>
+      <c r="G2" s="158"/>
       <c r="H2" s="160"/>
       <c r="I2" s="111" t="s">
         <v>36</v>
@@ -5325,16 +5334,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="O1:Q1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="O1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="K35:K1048576 K27:K32 K1:K25">
     <cfRule type="top10" dxfId="18" priority="9" percent="1" rank="25"/>
@@ -5381,10 +5390,10 @@
       <c r="C1" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="151" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -5402,22 +5411,22 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="181" t="s">
+      <c r="S1" s="162"/>
+      <c r="T1" s="178" t="s">
         <v>19</v>
       </c>
     </row>
@@ -5425,8 +5434,8 @@
       <c r="A2" s="154"/>
       <c r="B2" s="148"/>
       <c r="C2" s="171"/>
-      <c r="D2" s="150"/>
-      <c r="E2" s="152"/>
+      <c r="D2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="148"/>
       <c r="H2" s="148"/>
@@ -5475,10 +5484,10 @@
       <c r="D3" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="178">
-        <v>0</v>
-      </c>
-      <c r="F3" s="180">
+      <c r="E3" s="179">
+        <v>0</v>
+      </c>
+      <c r="F3" s="181">
         <v>0</v>
       </c>
       <c r="G3" s="58">
@@ -5530,8 +5539,8 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E4" s="179"/>
-      <c r="F4" s="172"/>
+      <c r="E4" s="180"/>
+      <c r="F4" s="174"/>
       <c r="G4" s="58">
         <v>35.6</v>
       </c>
@@ -5584,10 +5593,10 @@
       <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="173">
+      <c r="E5" s="172">
         <v>32.700000000000003</v>
       </c>
-      <c r="F5" s="174">
+      <c r="F5" s="173">
         <v>90.1</v>
       </c>
       <c r="G5" s="58">
@@ -5640,8 +5649,8 @@
       <c r="D6" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="173"/>
-      <c r="F6" s="174"/>
+      <c r="E6" s="172"/>
+      <c r="F6" s="173"/>
       <c r="G6" s="58">
         <v>35.6</v>
       </c>
@@ -5764,10 +5773,10 @@
       <c r="D9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="173">
+      <c r="E9" s="172">
         <v>66.599999999999994</v>
       </c>
-      <c r="F9" s="174">
+      <c r="F9" s="173">
         <v>181.3</v>
       </c>
       <c r="G9" s="58">
@@ -5819,8 +5828,8 @@
       <c r="D10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="173"/>
-      <c r="F10" s="174"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="173"/>
       <c r="G10" s="58">
         <v>75.8</v>
       </c>
@@ -5870,8 +5879,8 @@
       <c r="D11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="173"/>
-      <c r="F11" s="174"/>
+      <c r="E11" s="172"/>
+      <c r="F11" s="173"/>
       <c r="G11" s="58">
         <v>89.5</v>
       </c>
@@ -5919,8 +5928,8 @@
       <c r="D12" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="173"/>
-      <c r="F12" s="174"/>
+      <c r="E12" s="172"/>
+      <c r="F12" s="173"/>
       <c r="G12" s="58">
         <v>46.1</v>
       </c>
@@ -5970,8 +5979,8 @@
       <c r="D13" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="173"/>
-      <c r="F13" s="174"/>
+      <c r="E13" s="172"/>
+      <c r="F13" s="173"/>
       <c r="G13" s="58">
         <v>73.400000000000006</v>
       </c>
@@ -6020,8 +6029,8 @@
       <c r="D14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="173"/>
-      <c r="F14" s="174"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="173"/>
       <c r="G14" s="58">
         <v>88.4</v>
       </c>
@@ -6070,8 +6079,8 @@
       <c r="D15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="173"/>
-      <c r="F15" s="174"/>
+      <c r="E15" s="172"/>
+      <c r="F15" s="173"/>
       <c r="G15" s="58">
         <v>27.5</v>
       </c>
@@ -6120,8 +6129,8 @@
       <c r="D16" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="173"/>
-      <c r="F16" s="174"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="173"/>
       <c r="G16" s="58">
         <v>94.8</v>
       </c>
@@ -6170,8 +6179,8 @@
       <c r="D17" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="173"/>
-      <c r="F17" s="174"/>
+      <c r="E17" s="172"/>
+      <c r="F17" s="173"/>
       <c r="G17" s="58">
         <v>861.6</v>
       </c>
@@ -6223,8 +6232,8 @@
       <c r="D18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="173"/>
-      <c r="F18" s="174"/>
+      <c r="E18" s="172"/>
+      <c r="F18" s="173"/>
       <c r="G18" s="58">
         <v>48.1</v>
       </c>
@@ -6273,8 +6282,8 @@
       <c r="D19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="173"/>
-      <c r="F19" s="174"/>
+      <c r="E19" s="172"/>
+      <c r="F19" s="173"/>
       <c r="G19" s="58">
         <v>41.8</v>
       </c>
@@ -6329,14 +6338,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:P1"/>
     <mergeCell ref="E9:E19"/>
     <mergeCell ref="F9:F19"/>
     <mergeCell ref="B1:B2"/>
@@ -6351,6 +6352,14 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
@@ -6384,40 +6393,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="185" t="s">
+      <c r="B1" s="193" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="186" t="s">
+      <c r="C1" s="188" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="188" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="186" t="s">
+      <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="193" t="s">
+      <c r="F1" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="193"/>
-      <c r="H1" s="187" t="s">
+      <c r="G1" s="189"/>
+      <c r="H1" s="182" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="187"/>
-      <c r="J1" s="188" t="s">
+      <c r="I1" s="182"/>
+      <c r="J1" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="188"/>
+      <c r="K1" s="183"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="185"/>
-      <c r="B2" s="185"/>
-      <c r="C2" s="186"/>
-      <c r="D2" s="186"/>
-      <c r="E2" s="186"/>
+      <c r="A2" s="193"/>
+      <c r="B2" s="193"/>
+      <c r="C2" s="188"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="188"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -6438,16 +6447,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="189" t="s">
+      <c r="A3" s="184" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="189">
+      <c r="C3" s="184">
         <v>1550</v>
       </c>
-      <c r="D3" s="189" t="s">
+      <c r="D3" s="184" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="13">
@@ -6473,12 +6482,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="190"/>
+      <c r="A4" s="185"/>
       <c r="B4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="190"/>
-      <c r="D4" s="192"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="187"/>
       <c r="E4" s="18">
         <v>52</v>
       </c>
@@ -6502,11 +6511,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="190"/>
+      <c r="A5" s="185"/>
       <c r="B5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="190"/>
+      <c r="C5" s="185"/>
       <c r="D5" s="19" t="s">
         <v>14</v>
       </c>
@@ -6534,11 +6543,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="191"/>
+      <c r="A6" s="186"/>
       <c r="B6" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="191"/>
+      <c r="C6" s="186"/>
       <c r="D6" s="23" t="s">
         <v>15</v>
       </c>
@@ -6566,16 +6575,16 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="182" t="s">
+      <c r="A7" s="190" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="182">
+      <c r="C7" s="190">
         <v>1320</v>
       </c>
-      <c r="D7" s="182" t="s">
+      <c r="D7" s="190" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="3">
@@ -6601,12 +6610,12 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="183"/>
+      <c r="A8" s="191"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="183"/>
-      <c r="D8" s="184"/>
+      <c r="C8" s="191"/>
+      <c r="D8" s="192"/>
       <c r="E8" s="1">
         <v>100</v>
       </c>
@@ -6630,11 +6639,11 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="183"/>
+      <c r="A9" s="191"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="183"/>
+      <c r="C9" s="191"/>
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
@@ -6662,11 +6671,11 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="183"/>
+      <c r="A10" s="191"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="183"/>
+      <c r="C10" s="191"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
@@ -6694,11 +6703,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="184"/>
+      <c r="A11" s="192"/>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="184"/>
+      <c r="C11" s="192"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
@@ -6727,6 +6736,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="C3:C6"/>
@@ -6734,13 +6750,6 @@
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6759,40 +6768,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="185" t="s">
+      <c r="B1" s="193" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="186" t="s">
+      <c r="C1" s="188" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="188" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="186" t="s">
+      <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="193" t="s">
+      <c r="F1" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="193"/>
-      <c r="H1" s="187" t="s">
+      <c r="G1" s="189"/>
+      <c r="H1" s="182" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="187"/>
-      <c r="J1" s="188" t="s">
+      <c r="I1" s="182"/>
+      <c r="J1" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="188"/>
+      <c r="K1" s="183"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="185"/>
-      <c r="B2" s="185"/>
-      <c r="C2" s="186"/>
-      <c r="D2" s="186"/>
-      <c r="E2" s="186"/>
+      <c r="A2" s="193"/>
+      <c r="B2" s="193"/>
+      <c r="C2" s="188"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="188"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -6813,16 +6822,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="182" t="s">
+      <c r="A3" s="190" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="182">
+      <c r="C3" s="190">
         <v>1320</v>
       </c>
-      <c r="D3" s="182" t="s">
+      <c r="D3" s="190" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="3">
@@ -6848,12 +6857,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="183"/>
+      <c r="A4" s="191"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="183"/>
-      <c r="D4" s="184"/>
+      <c r="C4" s="191"/>
+      <c r="D4" s="192"/>
       <c r="E4" s="1">
         <v>100</v>
       </c>
@@ -6877,11 +6886,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="183"/>
+      <c r="A5" s="191"/>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="183"/>
+      <c r="C5" s="191"/>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
@@ -6909,11 +6918,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="183"/>
+      <c r="A6" s="191"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="183"/>
+      <c r="C6" s="191"/>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
@@ -6941,11 +6950,11 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="184"/>
+      <c r="A7" s="192"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="184"/>
+      <c r="C7" s="192"/>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
@@ -6992,7 +7001,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6C66A9-86C5-4B44-B720-CA86E494EFA2}">
-  <dimension ref="A1:W35"/>
+  <dimension ref="A1:Y35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
@@ -7017,17 +7026,17 @@
     <col min="24" max="16384" width="9.140625" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="147" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="149" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="151" t="s">
+      <c r="D1" s="161" t="s">
         <v>98</v>
       </c>
       <c r="E1" s="153" t="s">
@@ -7039,41 +7048,41 @@
       <c r="G1" s="155" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="162" t="s">
+      <c r="H1" s="157" t="s">
         <v>172</v>
       </c>
       <c r="I1" s="159" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="151" t="s">
+      <c r="J1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="K1" s="153"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="151" t="s">
+      <c r="L1" s="162"/>
+      <c r="M1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="N1" s="153"/>
-      <c r="O1" s="161"/>
-      <c r="P1" s="151" t="s">
+      <c r="O1" s="162"/>
+      <c r="P1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="153"/>
-      <c r="R1" s="161"/>
+      <c r="R1" s="162"/>
       <c r="T1" s="72"/>
       <c r="U1" s="72"/>
       <c r="V1" s="72"/>
       <c r="W1" s="128"/>
     </row>
-    <row r="2" spans="1:23" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="152"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="163"/>
       <c r="E2" s="154"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
-      <c r="H2" s="163"/>
+      <c r="H2" s="158"/>
       <c r="I2" s="160"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
@@ -7108,7 +7117,7 @@
       <c r="V2" s="144"/>
       <c r="W2" s="127"/>
     </row>
-    <row r="3" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
         <v>1064</v>
       </c>
@@ -7171,7 +7180,7 @@
       <c r="U3" s="69"/>
       <c r="V3" s="69"/>
     </row>
-    <row r="4" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="32" t="s">
         <v>124</v>
       </c>
@@ -7231,7 +7240,7 @@
       <c r="U4" s="69"/>
       <c r="V4" s="69"/>
     </row>
-    <row r="5" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="35"/>
       <c r="C5" s="38" t="s">
         <v>122</v>
@@ -7288,7 +7297,7 @@
       <c r="U5" s="69"/>
       <c r="V5" s="69"/>
     </row>
-    <row r="6" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35"/>
       <c r="C6" s="38" t="s">
         <v>125</v>
@@ -7343,7 +7352,7 @@
       <c r="U6" s="69"/>
       <c r="V6" s="69"/>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C7" s="81" t="s">
         <v>105</v>
       </c>
@@ -7395,7 +7404,7 @@
         <v>-0.154</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B8" s="71" t="s">
         <v>106</v>
       </c>
@@ -7458,8 +7467,11 @@
       <c r="V8" s="69" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X8" s="142" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B9" s="71" t="s">
         <v>106</v>
       </c>
@@ -7522,8 +7534,14 @@
       <c r="V9" s="35">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X9" s="32">
+        <v>1.3805000000000001</v>
+      </c>
+      <c r="Y9" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B10" s="71"/>
       <c r="D10" s="126"/>
       <c r="G10" s="84"/>
@@ -7541,7 +7559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C11" s="81" t="s">
         <v>126</v>
       </c>
@@ -7600,7 +7618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C12" s="38" t="s">
         <v>104</v>
       </c>
@@ -7661,7 +7679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="30"/>
       <c r="G13" s="84"/>
       <c r="H13" s="134"/>
@@ -7675,7 +7693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B14" s="35" t="s">
         <v>100</v>
       </c>
@@ -7738,8 +7756,14 @@
       <c r="V14" s="138">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X14" s="32">
+        <v>3.8134999999999999</v>
+      </c>
+      <c r="Y14" s="32">
+        <v>0.13181000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="30"/>
       <c r="B15" s="35" t="s">
         <v>100</v>
@@ -7804,8 +7828,14 @@
       <c r="V15" s="35">
         <v>9.7441000000000003E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X15" s="32">
+        <v>5.0713999999999997</v>
+      </c>
+      <c r="Y15" s="32">
+        <v>0.68649000000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B16" s="35" t="s">
         <v>100</v>
       </c>
@@ -7864,10 +7894,10 @@
         <v>135</v>
       </c>
       <c r="U16" s="35">
-        <v>3.9016999999999999</v>
-      </c>
-      <c r="V16" s="35">
-        <v>0</v>
+        <v>3.5552000000000001</v>
+      </c>
+      <c r="V16" s="35" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
@@ -7924,21 +7954,21 @@
       <c r="R17" s="90">
         <f>P17-Q17</f>
         <v>-4.9999999999999975E-3</v>
+      </c>
+      <c r="T17" s="35" t="s">
+        <v>178</v>
+      </c>
+      <c r="U17" s="35">
+        <v>3.9016999999999999</v>
+      </c>
+      <c r="V17" s="35">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="L18" s="90"/>
       <c r="O18" s="90"/>
       <c r="R18" s="90"/>
-      <c r="T18" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="U18" s="35">
-        <v>4.4375999999999998</v>
-      </c>
-      <c r="V18" s="35">
-        <v>0.49270599999999998</v>
-      </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="32">
@@ -7998,13 +8028,13 @@
         <v>-0.38300000000000001</v>
       </c>
       <c r="T19" s="35" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U19" s="35">
-        <v>6.0743999999999998</v>
+        <v>4.4375999999999998</v>
       </c>
       <c r="V19" s="35">
-        <v>2.4540289999999998</v>
+        <v>0.49270599999999998</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -8061,6 +8091,15 @@
         <f t="shared" si="6"/>
         <v>-0.7669999999999999</v>
       </c>
+      <c r="T20" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="U20" s="35">
+        <v>6.0743999999999998</v>
+      </c>
+      <c r="V20" s="35">
+        <v>2.4540289999999998</v>
+      </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B21" s="35" t="s">
@@ -8115,15 +8154,6 @@
         <f t="shared" si="6"/>
         <v>-0.8869999999999999</v>
       </c>
-      <c r="T21" s="35" t="s">
-        <v>175</v>
-      </c>
-      <c r="U21" s="35">
-        <v>2.7486000000000002</v>
-      </c>
-      <c r="V21" s="35">
-        <v>0.47835699999999998</v>
-      </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B22" s="35" t="s">
@@ -8179,13 +8209,13 @@
         <v>-0.90599999999999992</v>
       </c>
       <c r="T22" s="35" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U22" s="35">
-        <v>1.3346</v>
+        <v>2.7486000000000002</v>
       </c>
       <c r="V22" s="35">
-        <v>1.4580230000000001</v>
+        <v>0.47835699999999998</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
@@ -8240,6 +8270,15 @@
       <c r="R23" s="42">
         <f t="shared" si="6"/>
         <v>-0.91199999999999992</v>
+      </c>
+      <c r="T23" s="35" t="s">
+        <v>176</v>
+      </c>
+      <c r="U23" s="35">
+        <v>1.3346</v>
+      </c>
+      <c r="V23" s="35">
+        <v>1.4580230000000001</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
@@ -8794,11 +8833,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="H1:H2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
@@ -8806,12 +8840,18 @@
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="F1:F2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L1:L1048576">
     <cfRule type="top10" dxfId="17" priority="1" percent="1" rank="25"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8846,13 +8886,13 @@
       <c r="A1" s="147" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="149" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="151" t="s">
+      <c r="D1" s="161" t="s">
         <v>98</v>
       </c>
       <c r="E1" s="153" t="s">
@@ -8864,27 +8904,27 @@
       <c r="G1" s="155" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="162" t="s">
+      <c r="H1" s="157" t="s">
         <v>172</v>
       </c>
       <c r="I1" s="159" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="151" t="s">
+      <c r="J1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="K1" s="153"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="151" t="s">
+      <c r="L1" s="162"/>
+      <c r="M1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="N1" s="153"/>
-      <c r="O1" s="161"/>
-      <c r="P1" s="151" t="s">
+      <c r="O1" s="162"/>
+      <c r="P1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="153"/>
-      <c r="R1" s="161"/>
+      <c r="R1" s="162"/>
       <c r="S1" s="128"/>
       <c r="T1" s="69"/>
       <c r="U1" s="69"/>
@@ -8892,13 +8932,13 @@
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="152"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="163"/>
       <c r="E2" s="154"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
-      <c r="H2" s="163"/>
+      <c r="H2" s="158"/>
       <c r="I2" s="160"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
@@ -9710,13 +9750,13 @@
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="151" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -9734,21 +9774,21 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="S1" s="162"/>
       <c r="T1" s="147" t="s">
         <v>72</v>
       </c>
@@ -9756,8 +9796,8 @@
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="148"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="150"/>
-      <c r="E2" s="152"/>
+      <c r="C2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
       <c r="H2" s="166"/>
@@ -11062,6 +11102,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
@@ -11071,11 +11116,6 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <conditionalFormatting sqref="M1:M1048576">
     <cfRule type="top10" dxfId="14" priority="1" percent="1" rank="25"/>
@@ -11127,7 +11167,7 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -11145,21 +11185,21 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="S1" s="162"/>
       <c r="T1" s="147" t="s">
         <v>72</v>
       </c>
@@ -11168,7 +11208,7 @@
       <c r="A2" s="148"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
       <c r="H2" s="148"/>
@@ -12128,6 +12168,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -12136,12 +12182,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
@@ -12201,7 +12241,7 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -12219,21 +12259,21 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="S1" s="162"/>
       <c r="T1" s="147" t="s">
         <v>72</v>
       </c>
@@ -12242,7 +12282,7 @@
       <c r="A2" s="148"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
       <c r="H2" s="148"/>
@@ -12943,6 +12983,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -12951,12 +12997,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
     <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
@@ -13015,7 +13055,7 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -13033,21 +13073,21 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="S1" s="162"/>
       <c r="T1" s="147" t="s">
         <v>72</v>
       </c>
@@ -13056,7 +13096,7 @@
       <c r="A2" s="148"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
       <c r="H2" s="148"/>
@@ -13636,12 +13676,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -13650,6 +13684,12 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
@@ -13702,13 +13742,13 @@
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="151" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -13726,30 +13766,30 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="157" t="s">
+      <c r="S1" s="162"/>
+      <c r="T1" s="149" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="148"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="150"/>
-      <c r="E2" s="152"/>
+      <c r="C2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="156"/>
       <c r="H2" s="166"/>
@@ -13782,7 +13822,7 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="158"/>
+      <c r="T2" s="150"/>
       <c r="V2" s="154"/>
       <c r="W2" s="154"/>
       <c r="X2" s="154"/>
@@ -15026,6 +15066,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -15034,12 +15080,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
@@ -15105,10 +15145,10 @@
       <c r="C1" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="151" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="161" t="s">
         <v>30</v>
       </c>
       <c r="F1" s="153" t="s">
@@ -15126,21 +15166,21 @@
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="161" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="M1" s="162"/>
+      <c r="N1" s="161" t="s">
         <v>4</v>
       </c>
       <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="161" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="S1" s="162"/>
       <c r="T1" s="176" t="s">
         <v>19</v>
       </c>
@@ -15149,8 +15189,8 @@
       <c r="A2" s="154"/>
       <c r="B2" s="148"/>
       <c r="C2" s="171"/>
-      <c r="D2" s="150"/>
-      <c r="E2" s="152"/>
+      <c r="D2" s="152"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="154"/>
       <c r="G2" s="148"/>
       <c r="H2" s="148"/>
@@ -15257,10 +15297,10 @@
       <c r="D4" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="173">
+      <c r="E4" s="172">
         <v>32.700000000000003</v>
       </c>
-      <c r="F4" s="174">
+      <c r="F4" s="173">
         <v>90.1</v>
       </c>
       <c r="G4" s="175">
@@ -15309,12 +15349,12 @@
       <c r="D5" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="173"/>
-      <c r="F5" s="174"/>
-      <c r="G5" s="172">
+      <c r="E5" s="172"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="174">
         <v>41.2</v>
       </c>
-      <c r="H5" s="172"/>
+      <c r="H5" s="174"/>
       <c r="I5" s="58">
         <v>15.1</v>
       </c>
@@ -15359,12 +15399,12 @@
       <c r="D6" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="173"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="172">
+      <c r="E6" s="172"/>
+      <c r="F6" s="173"/>
+      <c r="G6" s="174">
         <v>24.3</v>
       </c>
-      <c r="H6" s="172"/>
+      <c r="H6" s="174"/>
       <c r="I6" s="58">
         <v>30.6</v>
       </c>
@@ -15406,12 +15446,12 @@
       <c r="D7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="173"/>
-      <c r="F7" s="174"/>
-      <c r="G7" s="172">
+      <c r="E7" s="172"/>
+      <c r="F7" s="173"/>
+      <c r="G7" s="174">
         <v>42.6</v>
       </c>
-      <c r="H7" s="172"/>
+      <c r="H7" s="174"/>
       <c r="I7" s="58">
         <v>13.3</v>
       </c>
@@ -15455,12 +15495,12 @@
       <c r="D8" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="173"/>
-      <c r="F8" s="174"/>
-      <c r="G8" s="172">
+      <c r="E8" s="172"/>
+      <c r="F8" s="173"/>
+      <c r="G8" s="174">
         <v>31.9</v>
       </c>
-      <c r="H8" s="172"/>
+      <c r="H8" s="174"/>
       <c r="I8" s="58">
         <v>23.7</v>
       </c>
@@ -15502,8 +15542,8 @@
       <c r="D9" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="173"/>
-      <c r="F9" s="174"/>
+      <c r="E9" s="172"/>
+      <c r="F9" s="173"/>
       <c r="G9" s="66">
         <v>2.7</v>
       </c>
@@ -15552,8 +15592,8 @@
       <c r="D10" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="173"/>
-      <c r="F10" s="174"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="173"/>
       <c r="G10" s="58">
         <v>4.2</v>
       </c>
@@ -15602,8 +15642,8 @@
       <c r="D11" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="173"/>
-      <c r="F11" s="174"/>
+      <c r="E11" s="172"/>
+      <c r="F11" s="173"/>
       <c r="G11" s="58">
         <v>1.3</v>
       </c>
@@ -15721,16 +15761,16 @@
       <c r="D14" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="173">
+      <c r="E14" s="172">
         <v>66.599999999999994</v>
       </c>
-      <c r="F14" s="174">
+      <c r="F14" s="173">
         <v>181.3</v>
       </c>
-      <c r="G14" s="172">
+      <c r="G14" s="174">
         <v>107.3</v>
       </c>
-      <c r="H14" s="172"/>
+      <c r="H14" s="174"/>
       <c r="I14" s="58">
         <v>0</v>
       </c>
@@ -15772,8 +15812,8 @@
       <c r="D15" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="173"/>
-      <c r="F15" s="174"/>
+      <c r="E15" s="172"/>
+      <c r="F15" s="173"/>
       <c r="G15" s="175">
         <v>68.7</v>
       </c>
@@ -15820,8 +15860,8 @@
       <c r="D16" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="173"/>
-      <c r="F16" s="174"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="173"/>
       <c r="G16" s="175">
         <v>105</v>
       </c>
@@ -15868,12 +15908,12 @@
       <c r="D17" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="173"/>
-      <c r="F17" s="174"/>
-      <c r="G17" s="172">
+      <c r="E17" s="172"/>
+      <c r="F17" s="173"/>
+      <c r="G17" s="174">
         <v>65.599999999999994</v>
       </c>
-      <c r="H17" s="172"/>
+      <c r="H17" s="174"/>
       <c r="I17" s="58">
         <v>53.5</v>
       </c>
@@ -15916,8 +15956,8 @@
       <c r="D18" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="173"/>
-      <c r="F18" s="174"/>
+      <c r="E18" s="172"/>
+      <c r="F18" s="173"/>
       <c r="G18" s="58">
         <v>42.6</v>
       </c>
@@ -15966,8 +16006,8 @@
       <c r="D19" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="173"/>
-      <c r="F19" s="174"/>
+      <c r="E19" s="172"/>
+      <c r="F19" s="173"/>
       <c r="G19" s="58">
         <v>47.7</v>
       </c>
@@ -16016,8 +16056,8 @@
       <c r="D20" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="173"/>
-      <c r="F20" s="174"/>
+      <c r="E20" s="172"/>
+      <c r="F20" s="173"/>
       <c r="G20" s="58">
         <v>48.7</v>
       </c>
@@ -16173,12 +16213,18 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="E14:E20"/>
-    <mergeCell ref="F14:F20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E4:E11"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -16190,18 +16236,12 @@
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E4:E11"/>
-    <mergeCell ref="F4:F11"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E14:E20"/>
+    <mergeCell ref="F14:F20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">

</xml_diff>

<commit_message>
Add comparison table to IV.D.
</commit_message>
<xml_diff>
--- a/AsymReca_ThkCalc.xlsb.xlsx
+++ b/AsymReca_ThkCalc.xlsb.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2024-ILLUSTRIOUS\My Drive (61050734@kmitl.ac.th)\AsymReca_SbSe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4674DA89-5D02-4A35-B75C-A29EA1025E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DF4A9B-9C8B-423E-A66E-BF83F82CB02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="-120" windowWidth="28200" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22965" yWindow="5385" windowWidth="20970" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532_back" sheetId="15" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="184">
   <si>
     <t>Wavelength (nm)</t>
   </si>
@@ -2181,6 +2181,12 @@
   </si>
   <si>
     <t>N2 SbSe N2</t>
+  </si>
+  <si>
+    <t>Design of near-infrared solid-state tunable Fabry-Perot filters based on VO2-P4VP films</t>
+  </si>
+  <si>
+    <t>2 DBR paris, 4% vol. frac.</t>
   </si>
 </sst>
 </file>
@@ -2555,7 +2561,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="196">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2993,6 +2999,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3005,15 +3032,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3029,21 +3050,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3068,15 +3074,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -3086,6 +3092,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -3095,8 +3104,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3110,29 +3140,11 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3630,59 +3642,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="162" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="156" t="s">
         <v>121</v>
       </c>
       <c r="D1" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="153" t="s">
+      <c r="E1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="155" t="s">
+      <c r="F1" s="160" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="162" t="s">
+      <c r="G1" s="152" t="s">
         <v>116</v>
       </c>
-      <c r="H1" s="159" t="s">
+      <c r="H1" s="147" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="151" t="s">
+      <c r="I1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="153"/>
-      <c r="K1" s="161"/>
-      <c r="L1" s="151" t="s">
+      <c r="J1" s="150"/>
+      <c r="K1" s="151"/>
+      <c r="L1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="153"/>
-      <c r="N1" s="161"/>
-      <c r="O1" s="151" t="s">
+      <c r="M1" s="150"/>
+      <c r="N1" s="151"/>
+      <c r="O1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="153"/>
-      <c r="Q1" s="161"/>
+      <c r="P1" s="150"/>
+      <c r="Q1" s="151"/>
       <c r="S1" s="128"/>
       <c r="T1" s="128"/>
       <c r="U1" s="128"/>
       <c r="V1" s="128"/>
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
+      <c r="A2" s="155"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="157"/>
       <c r="D2" s="44"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="163"/>
-      <c r="H2" s="160"/>
+      <c r="E2" s="159"/>
+      <c r="F2" s="161"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="148"/>
       <c r="I2" s="111" t="s">
         <v>36</v>
       </c>
@@ -5337,16 +5349,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="O1:Q1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="O1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="K35:K1048576 K27:K32 K1:K25">
     <cfRule type="top10" dxfId="18" priority="9" percent="1" rank="25"/>
@@ -5387,19 +5399,19 @@
       <c r="A1" s="176" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="147" t="s">
+      <c r="B1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="156" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
       <c r="G1" s="169" t="s">
@@ -5408,41 +5420,41 @@
       <c r="H1" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="181" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="178" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="154"/>
-      <c r="B2" s="148"/>
+      <c r="A2" s="159"/>
+      <c r="B2" s="155"/>
       <c r="C2" s="171"/>
-      <c r="D2" s="150"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="148"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="154"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
@@ -5472,10 +5484,10 @@
         <v>51</v>
       </c>
       <c r="T2" s="164"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="30">
@@ -5487,10 +5499,10 @@
       <c r="D3" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="178">
-        <v>0</v>
-      </c>
-      <c r="F3" s="180">
+      <c r="E3" s="179">
+        <v>0</v>
+      </c>
+      <c r="F3" s="181">
         <v>0</v>
       </c>
       <c r="G3" s="58">
@@ -5542,8 +5554,8 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E4" s="179"/>
-      <c r="F4" s="172"/>
+      <c r="E4" s="180"/>
+      <c r="F4" s="174"/>
       <c r="G4" s="58">
         <v>35.6</v>
       </c>
@@ -5596,10 +5608,10 @@
       <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="173">
+      <c r="E5" s="172">
         <v>32.700000000000003</v>
       </c>
-      <c r="F5" s="174">
+      <c r="F5" s="173">
         <v>90.1</v>
       </c>
       <c r="G5" s="58">
@@ -5652,8 +5664,8 @@
       <c r="D6" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="173"/>
-      <c r="F6" s="174"/>
+      <c r="E6" s="172"/>
+      <c r="F6" s="173"/>
       <c r="G6" s="58">
         <v>35.6</v>
       </c>
@@ -5776,10 +5788,10 @@
       <c r="D9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="173">
+      <c r="E9" s="172">
         <v>66.599999999999994</v>
       </c>
-      <c r="F9" s="174">
+      <c r="F9" s="173">
         <v>181.3</v>
       </c>
       <c r="G9" s="58">
@@ -5831,8 +5843,8 @@
       <c r="D10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="173"/>
-      <c r="F10" s="174"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="173"/>
       <c r="G10" s="58">
         <v>75.8</v>
       </c>
@@ -5882,8 +5894,8 @@
       <c r="D11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="173"/>
-      <c r="F11" s="174"/>
+      <c r="E11" s="172"/>
+      <c r="F11" s="173"/>
       <c r="G11" s="58">
         <v>89.5</v>
       </c>
@@ -5931,8 +5943,8 @@
       <c r="D12" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="173"/>
-      <c r="F12" s="174"/>
+      <c r="E12" s="172"/>
+      <c r="F12" s="173"/>
       <c r="G12" s="58">
         <v>46.1</v>
       </c>
@@ -5982,8 +5994,8 @@
       <c r="D13" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="173"/>
-      <c r="F13" s="174"/>
+      <c r="E13" s="172"/>
+      <c r="F13" s="173"/>
       <c r="G13" s="58">
         <v>73.400000000000006</v>
       </c>
@@ -6032,8 +6044,8 @@
       <c r="D14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="173"/>
-      <c r="F14" s="174"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="173"/>
       <c r="G14" s="58">
         <v>88.4</v>
       </c>
@@ -6082,8 +6094,8 @@
       <c r="D15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="173"/>
-      <c r="F15" s="174"/>
+      <c r="E15" s="172"/>
+      <c r="F15" s="173"/>
       <c r="G15" s="58">
         <v>27.5</v>
       </c>
@@ -6132,8 +6144,8 @@
       <c r="D16" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="173"/>
-      <c r="F16" s="174"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="173"/>
       <c r="G16" s="58">
         <v>94.8</v>
       </c>
@@ -6182,8 +6194,8 @@
       <c r="D17" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="173"/>
-      <c r="F17" s="174"/>
+      <c r="E17" s="172"/>
+      <c r="F17" s="173"/>
       <c r="G17" s="58">
         <v>861.6</v>
       </c>
@@ -6235,8 +6247,8 @@
       <c r="D18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="173"/>
-      <c r="F18" s="174"/>
+      <c r="E18" s="172"/>
+      <c r="F18" s="173"/>
       <c r="G18" s="58">
         <v>48.1</v>
       </c>
@@ -6285,8 +6297,8 @@
       <c r="D19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="173"/>
-      <c r="F19" s="174"/>
+      <c r="E19" s="172"/>
+      <c r="F19" s="173"/>
       <c r="G19" s="58">
         <v>41.8</v>
       </c>
@@ -6341,14 +6353,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:P1"/>
     <mergeCell ref="E9:E19"/>
     <mergeCell ref="F9:F19"/>
     <mergeCell ref="B1:B2"/>
@@ -6363,6 +6367,14 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
@@ -6396,40 +6408,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="185" t="s">
+      <c r="B1" s="193" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="186" t="s">
+      <c r="C1" s="188" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="188" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="186" t="s">
+      <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="193" t="s">
+      <c r="F1" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="193"/>
-      <c r="H1" s="187" t="s">
+      <c r="G1" s="189"/>
+      <c r="H1" s="182" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="187"/>
-      <c r="J1" s="188" t="s">
+      <c r="I1" s="182"/>
+      <c r="J1" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="188"/>
+      <c r="K1" s="183"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="185"/>
-      <c r="B2" s="185"/>
-      <c r="C2" s="186"/>
-      <c r="D2" s="186"/>
-      <c r="E2" s="186"/>
+      <c r="A2" s="193"/>
+      <c r="B2" s="193"/>
+      <c r="C2" s="188"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="188"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -6450,16 +6462,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="189" t="s">
+      <c r="A3" s="184" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="189">
+      <c r="C3" s="184">
         <v>1550</v>
       </c>
-      <c r="D3" s="189" t="s">
+      <c r="D3" s="184" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="13">
@@ -6485,12 +6497,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="190"/>
+      <c r="A4" s="185"/>
       <c r="B4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="190"/>
-      <c r="D4" s="192"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="187"/>
       <c r="E4" s="18">
         <v>52</v>
       </c>
@@ -6514,11 +6526,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="190"/>
+      <c r="A5" s="185"/>
       <c r="B5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="190"/>
+      <c r="C5" s="185"/>
       <c r="D5" s="19" t="s">
         <v>14</v>
       </c>
@@ -6546,11 +6558,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="191"/>
+      <c r="A6" s="186"/>
       <c r="B6" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="191"/>
+      <c r="C6" s="186"/>
       <c r="D6" s="23" t="s">
         <v>15</v>
       </c>
@@ -6578,16 +6590,16 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="182" t="s">
+      <c r="A7" s="190" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="182">
+      <c r="C7" s="190">
         <v>1320</v>
       </c>
-      <c r="D7" s="182" t="s">
+      <c r="D7" s="190" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="3">
@@ -6613,12 +6625,12 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="183"/>
+      <c r="A8" s="191"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="183"/>
-      <c r="D8" s="184"/>
+      <c r="C8" s="191"/>
+      <c r="D8" s="192"/>
       <c r="E8" s="1">
         <v>100</v>
       </c>
@@ -6642,11 +6654,11 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="183"/>
+      <c r="A9" s="191"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="183"/>
+      <c r="C9" s="191"/>
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
@@ -6674,11 +6686,11 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="183"/>
+      <c r="A10" s="191"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="183"/>
+      <c r="C10" s="191"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
@@ -6706,11 +6718,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="184"/>
+      <c r="A11" s="192"/>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="184"/>
+      <c r="C11" s="192"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
@@ -6739,6 +6751,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="C3:C6"/>
@@ -6746,13 +6765,6 @@
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6771,40 +6783,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="185" t="s">
+      <c r="B1" s="193" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="186" t="s">
+      <c r="C1" s="188" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="188" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="186" t="s">
+      <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="193" t="s">
+      <c r="F1" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="193"/>
-      <c r="H1" s="187" t="s">
+      <c r="G1" s="189"/>
+      <c r="H1" s="182" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="187"/>
-      <c r="J1" s="188" t="s">
+      <c r="I1" s="182"/>
+      <c r="J1" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="188"/>
+      <c r="K1" s="183"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="185"/>
-      <c r="B2" s="185"/>
-      <c r="C2" s="186"/>
-      <c r="D2" s="186"/>
-      <c r="E2" s="186"/>
+      <c r="A2" s="193"/>
+      <c r="B2" s="193"/>
+      <c r="C2" s="188"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="188"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -6825,16 +6837,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="182" t="s">
+      <c r="A3" s="190" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="182">
+      <c r="C3" s="190">
         <v>1320</v>
       </c>
-      <c r="D3" s="182" t="s">
+      <c r="D3" s="190" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="3">
@@ -6860,12 +6872,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="183"/>
+      <c r="A4" s="191"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="183"/>
-      <c r="D4" s="184"/>
+      <c r="C4" s="191"/>
+      <c r="D4" s="192"/>
       <c r="E4" s="1">
         <v>100</v>
       </c>
@@ -6889,11 +6901,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="183"/>
+      <c r="A5" s="191"/>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="183"/>
+      <c r="C5" s="191"/>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
@@ -6921,11 +6933,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="183"/>
+      <c r="A6" s="191"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="183"/>
+      <c r="C6" s="191"/>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
@@ -6953,11 +6965,11 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="184"/>
+      <c r="A7" s="192"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="184"/>
+      <c r="C7" s="192"/>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
@@ -7004,12 +7016,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6C66A9-86C5-4B44-B720-CA86E494EFA2}">
-  <dimension ref="A1:Y36"/>
+  <dimension ref="A1:Y45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" style="35" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" style="38" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" style="44" customWidth="1"/>
     <col min="5" max="7" width="7.7109375" style="34" customWidth="1"/>
     <col min="8" max="8" width="8.7109375" style="137" customWidth="1"/>
@@ -7030,63 +7042,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="162" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="156" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="151" t="s">
+      <c r="D1" s="149" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="153" t="s">
+      <c r="E1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="162" t="s">
+      <c r="H1" s="152" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="159" t="s">
+      <c r="I1" s="147" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="151" t="s">
+      <c r="J1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="153"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="151" t="s">
+      <c r="K1" s="150"/>
+      <c r="L1" s="151"/>
+      <c r="M1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="153"/>
-      <c r="O1" s="161"/>
-      <c r="P1" s="151" t="s">
+      <c r="N1" s="150"/>
+      <c r="O1" s="151"/>
+      <c r="P1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="153"/>
-      <c r="R1" s="161"/>
+      <c r="Q1" s="150"/>
+      <c r="R1" s="151"/>
       <c r="T1" s="72"/>
       <c r="U1" s="72"/>
       <c r="V1" s="72"/>
       <c r="W1" s="128"/>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="163"/>
-      <c r="I2" s="160"/>
+      <c r="A2" s="155"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="159"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="148"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
       </c>
@@ -8471,7 +8483,7 @@
         <v>99.9</v>
       </c>
       <c r="H28" s="137">
-        <f>G28</f>
+        <f t="shared" ref="H28:H33" si="7">G28</f>
         <v>99.9</v>
       </c>
       <c r="I28" s="136">
@@ -8484,7 +8496,7 @@
         <v>0.51200000000000001</v>
       </c>
       <c r="L28" s="90">
-        <f t="shared" ref="L28:L36" si="7">J28-K28</f>
+        <f t="shared" ref="L28:L36" si="8">J28-K28</f>
         <v>0.42300000000000004</v>
       </c>
       <c r="M28" s="92">
@@ -8504,7 +8516,7 @@
         <v>0.47499999999999998</v>
       </c>
       <c r="R28" s="90">
-        <f t="shared" ref="R28:R36" si="8">P28-Q28</f>
+        <f t="shared" ref="R28:R36" si="9">P28-Q28</f>
         <v>-0.41</v>
       </c>
     </row>
@@ -8525,7 +8537,7 @@
         <v>100</v>
       </c>
       <c r="H29" s="137">
-        <f>G29</f>
+        <f t="shared" si="7"/>
         <v>100</v>
       </c>
       <c r="I29" s="136">
@@ -8538,7 +8550,7 @@
         <v>0.27100000000000002</v>
       </c>
       <c r="L29" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.624</v>
       </c>
       <c r="M29" s="92">
@@ -8558,7 +8570,7 @@
         <v>0.71299999999999997</v>
       </c>
       <c r="R29" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.60799999999999998</v>
       </c>
     </row>
@@ -8579,7 +8591,7 @@
         <v>97.7</v>
       </c>
       <c r="H30" s="137">
-        <f>G30</f>
+        <f t="shared" si="7"/>
         <v>97.7</v>
       </c>
       <c r="I30" s="136">
@@ -8609,7 +8621,7 @@
         <v>31.6</v>
       </c>
       <c r="H31" s="137">
-        <f>G31</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I31" s="136">
@@ -8622,7 +8634,7 @@
         <v>0.83699999999999997</v>
       </c>
       <c r="L31" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.129</v>
       </c>
       <c r="M31" s="92">
@@ -8642,7 +8654,7 @@
         <v>0.155</v>
       </c>
       <c r="R31" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.121</v>
       </c>
     </row>
@@ -8663,7 +8675,7 @@
         <v>31.9</v>
       </c>
       <c r="H32" s="137">
-        <f>G32</f>
+        <f t="shared" si="7"/>
         <v>31.9</v>
       </c>
       <c r="I32" s="136">
@@ -8676,7 +8688,7 @@
         <v>0.498</v>
       </c>
       <c r="L32" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.46799999999999997</v>
       </c>
       <c r="M32" s="92">
@@ -8696,11 +8708,11 @@
         <v>0.49</v>
       </c>
       <c r="R32" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.45599999999999996</v>
       </c>
     </row>
-    <row r="33" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C33" s="81" t="s">
         <v>165</v>
       </c>
@@ -8717,7 +8729,7 @@
         <v>32</v>
       </c>
       <c r="H33" s="137">
-        <f>G33</f>
+        <f t="shared" si="7"/>
         <v>32</v>
       </c>
       <c r="I33" s="136">
@@ -8730,7 +8742,7 @@
         <v>0.11700000000000001</v>
       </c>
       <c r="L33" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.84799999999999998</v>
       </c>
       <c r="M33" s="92">
@@ -8750,11 +8762,11 @@
         <v>0.875</v>
       </c>
       <c r="R33" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.84</v>
       </c>
     </row>
-    <row r="35" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C35" s="37" t="s">
         <v>168</v>
       </c>
@@ -8782,7 +8794,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="L35" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.29599999999999999</v>
       </c>
       <c r="M35" s="92">
@@ -8802,11 +8814,11 @@
         <v>0.57399999999999995</v>
       </c>
       <c r="R35" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.36499999999999999</v>
       </c>
     </row>
-    <row r="36" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C36" s="146" t="s">
         <v>174</v>
       </c>
@@ -8834,7 +8846,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
       <c r="L36" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.21300000000000002</v>
       </c>
       <c r="M36" s="92">
@@ -8854,17 +8866,50 @@
         <v>0.315</v>
       </c>
       <c r="R36" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.16200000000000001</v>
       </c>
     </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" s="194" t="s">
+        <v>182</v>
+      </c>
+      <c r="B43" s="195"/>
+      <c r="C43" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="D43" s="44">
+        <f>1064/(4*2.299)</f>
+        <v>115.70247933884298</v>
+      </c>
+      <c r="E43" s="34">
+        <f>1064/(4*1.434)</f>
+        <v>185.49511854951186</v>
+      </c>
+      <c r="G43" s="34">
+        <f>1064/1.555</f>
+        <v>684.24437299035378</v>
+      </c>
+      <c r="H43" s="137">
+        <f>G43</f>
+        <v>684.24437299035378</v>
+      </c>
+      <c r="I43" s="136">
+        <f>2*2*(D43+E43)+G43</f>
+        <v>1889.0347645437732</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" s="194"/>
+      <c r="B44" s="195"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A45" s="194"/>
+      <c r="B45" s="195"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="H1:H2"/>
+  <mergeCells count="13">
+    <mergeCell ref="A43:B45"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
@@ -8872,6 +8917,11 @@
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="F1:F2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L1:L1048576">
@@ -8910,63 +8960,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="162" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="156" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="151" t="s">
+      <c r="D1" s="149" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="153" t="s">
+      <c r="E1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="162" t="s">
+      <c r="H1" s="152" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="159" t="s">
+      <c r="I1" s="147" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="151" t="s">
+      <c r="J1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="153"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="151" t="s">
+      <c r="K1" s="150"/>
+      <c r="L1" s="151"/>
+      <c r="M1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="153"/>
-      <c r="O1" s="161"/>
-      <c r="P1" s="151" t="s">
+      <c r="N1" s="150"/>
+      <c r="O1" s="151"/>
+      <c r="P1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="153"/>
-      <c r="R1" s="161"/>
+      <c r="Q1" s="150"/>
+      <c r="R1" s="151"/>
       <c r="S1" s="128"/>
       <c r="T1" s="69"/>
       <c r="U1" s="69"/>
       <c r="V1" s="69"/>
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
-      <c r="B2" s="158"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="163"/>
-      <c r="I2" s="160"/>
+      <c r="A2" s="155"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="159"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="148"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
       </c>
@@ -9771,64 +9821,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="156" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="165" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="147" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="154" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
+      <c r="A2" s="155"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="150"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
       <c r="H2" s="166"/>
-      <c r="I2" s="154"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
@@ -9857,11 +9907,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="148"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="155"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -11129,6 +11179,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
@@ -11138,11 +11193,6 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <conditionalFormatting sqref="M1:M1048576">
     <cfRule type="top10" dxfId="14" priority="1" percent="1" rank="25"/>
@@ -11182,7 +11232,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
@@ -11194,52 +11244,52 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="147" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="154" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
+      <c r="A2" s="155"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="154"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
@@ -11268,11 +11318,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="148"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="155"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -12195,6 +12245,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -12203,12 +12259,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
@@ -12256,7 +12306,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
@@ -12268,52 +12318,52 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="147" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="154" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
+      <c r="A2" s="155"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="154"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
@@ -12342,11 +12392,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="148"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="155"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -13010,6 +13060,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -13018,12 +13074,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
     <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
@@ -13070,7 +13120,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
@@ -13082,52 +13132,52 @@
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="147" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="154" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
+      <c r="A2" s="155"/>
       <c r="B2" s="115"/>
       <c r="C2" s="171"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="154"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
@@ -13156,11 +13206,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="148"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="155"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -13703,12 +13753,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -13717,6 +13761,12 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
@@ -13763,64 +13813,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="156" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="160" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="165" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
-      <c r="T1" s="157" t="s">
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="162" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="148"/>
+      <c r="A2" s="155"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="150"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="161"/>
       <c r="H2" s="166"/>
-      <c r="I2" s="154"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
@@ -13849,11 +13899,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="158"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="163"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -15093,6 +15143,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -15101,12 +15157,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
@@ -15166,19 +15216,19 @@
       <c r="A1" s="176" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="147" t="s">
+      <c r="B1" s="154" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="156" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="151" t="s">
+      <c r="E1" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="153" t="s">
+      <c r="F1" s="150" t="s">
         <v>29</v>
       </c>
       <c r="G1" s="169" t="s">
@@ -15187,41 +15237,41 @@
       <c r="H1" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="150" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="151" t="s">
+      <c r="K1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="153"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="151" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="153"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="151" t="s">
+      <c r="O1" s="150"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="153"/>
-      <c r="S1" s="161"/>
+      <c r="R1" s="150"/>
+      <c r="S1" s="151"/>
       <c r="T1" s="176" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="154"/>
-      <c r="B2" s="148"/>
+      <c r="A2" s="159"/>
+      <c r="B2" s="155"/>
       <c r="C2" s="171"/>
-      <c r="D2" s="150"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="148"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="154"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="159"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="159"/>
       <c r="J2" s="168"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
@@ -15250,11 +15300,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="154"/>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
+      <c r="T2" s="159"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="46">
@@ -15324,10 +15374,10 @@
       <c r="D4" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="173">
+      <c r="E4" s="172">
         <v>32.700000000000003</v>
       </c>
-      <c r="F4" s="174">
+      <c r="F4" s="173">
         <v>90.1</v>
       </c>
       <c r="G4" s="175">
@@ -15376,12 +15426,12 @@
       <c r="D5" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="173"/>
-      <c r="F5" s="174"/>
-      <c r="G5" s="172">
+      <c r="E5" s="172"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="174">
         <v>41.2</v>
       </c>
-      <c r="H5" s="172"/>
+      <c r="H5" s="174"/>
       <c r="I5" s="58">
         <v>15.1</v>
       </c>
@@ -15426,12 +15476,12 @@
       <c r="D6" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="173"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="172">
+      <c r="E6" s="172"/>
+      <c r="F6" s="173"/>
+      <c r="G6" s="174">
         <v>24.3</v>
       </c>
-      <c r="H6" s="172"/>
+      <c r="H6" s="174"/>
       <c r="I6" s="58">
         <v>30.6</v>
       </c>
@@ -15473,12 +15523,12 @@
       <c r="D7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="173"/>
-      <c r="F7" s="174"/>
-      <c r="G7" s="172">
+      <c r="E7" s="172"/>
+      <c r="F7" s="173"/>
+      <c r="G7" s="174">
         <v>42.6</v>
       </c>
-      <c r="H7" s="172"/>
+      <c r="H7" s="174"/>
       <c r="I7" s="58">
         <v>13.3</v>
       </c>
@@ -15522,12 +15572,12 @@
       <c r="D8" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="173"/>
-      <c r="F8" s="174"/>
-      <c r="G8" s="172">
+      <c r="E8" s="172"/>
+      <c r="F8" s="173"/>
+      <c r="G8" s="174">
         <v>31.9</v>
       </c>
-      <c r="H8" s="172"/>
+      <c r="H8" s="174"/>
       <c r="I8" s="58">
         <v>23.7</v>
       </c>
@@ -15569,8 +15619,8 @@
       <c r="D9" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="173"/>
-      <c r="F9" s="174"/>
+      <c r="E9" s="172"/>
+      <c r="F9" s="173"/>
       <c r="G9" s="66">
         <v>2.7</v>
       </c>
@@ -15619,8 +15669,8 @@
       <c r="D10" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="173"/>
-      <c r="F10" s="174"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="173"/>
       <c r="G10" s="58">
         <v>4.2</v>
       </c>
@@ -15669,8 +15719,8 @@
       <c r="D11" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="173"/>
-      <c r="F11" s="174"/>
+      <c r="E11" s="172"/>
+      <c r="F11" s="173"/>
       <c r="G11" s="58">
         <v>1.3</v>
       </c>
@@ -15788,16 +15838,16 @@
       <c r="D14" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="173">
+      <c r="E14" s="172">
         <v>66.599999999999994</v>
       </c>
-      <c r="F14" s="174">
+      <c r="F14" s="173">
         <v>181.3</v>
       </c>
-      <c r="G14" s="172">
+      <c r="G14" s="174">
         <v>107.3</v>
       </c>
-      <c r="H14" s="172"/>
+      <c r="H14" s="174"/>
       <c r="I14" s="58">
         <v>0</v>
       </c>
@@ -15839,8 +15889,8 @@
       <c r="D15" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="173"/>
-      <c r="F15" s="174"/>
+      <c r="E15" s="172"/>
+      <c r="F15" s="173"/>
       <c r="G15" s="175">
         <v>68.7</v>
       </c>
@@ -15887,8 +15937,8 @@
       <c r="D16" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="173"/>
-      <c r="F16" s="174"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="173"/>
       <c r="G16" s="175">
         <v>105</v>
       </c>
@@ -15935,12 +15985,12 @@
       <c r="D17" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="173"/>
-      <c r="F17" s="174"/>
-      <c r="G17" s="172">
+      <c r="E17" s="172"/>
+      <c r="F17" s="173"/>
+      <c r="G17" s="174">
         <v>65.599999999999994</v>
       </c>
-      <c r="H17" s="172"/>
+      <c r="H17" s="174"/>
       <c r="I17" s="58">
         <v>53.5</v>
       </c>
@@ -15983,8 +16033,8 @@
       <c r="D18" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="173"/>
-      <c r="F18" s="174"/>
+      <c r="E18" s="172"/>
+      <c r="F18" s="173"/>
       <c r="G18" s="58">
         <v>42.6</v>
       </c>
@@ -16033,8 +16083,8 @@
       <c r="D19" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="173"/>
-      <c r="F19" s="174"/>
+      <c r="E19" s="172"/>
+      <c r="F19" s="173"/>
       <c r="G19" s="58">
         <v>47.7</v>
       </c>
@@ -16083,8 +16133,8 @@
       <c r="D20" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="173"/>
-      <c r="F20" s="174"/>
+      <c r="E20" s="172"/>
+      <c r="F20" s="173"/>
       <c r="G20" s="58">
         <v>48.7</v>
       </c>
@@ -16240,12 +16290,18 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="E14:E20"/>
-    <mergeCell ref="F14:F20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E4:E11"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -16257,18 +16313,12 @@
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E4:E11"/>
-    <mergeCell ref="F4:F11"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E14:E20"/>
+    <mergeCell ref="F14:F20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">

</xml_diff>

<commit_message>
Add limitation & future works
</commit_message>
<xml_diff>
--- a/AsymReca_ThkCalc.xlsb.xlsx
+++ b/AsymReca_ThkCalc.xlsb.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DF4A9B-9C8B-423E-A66E-BF83F82CB02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22965" yWindow="5385" windowWidth="20970" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532_back" sheetId="15" r:id="rId1"/>
@@ -2999,18 +2999,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3020,36 +3056,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3074,15 +3080,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -3092,17 +3098,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3122,29 +3143,8 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3642,59 +3642,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="162" t="s">
+      <c r="B1" s="159" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
       <c r="D1" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="150" t="s">
+      <c r="E1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="160" t="s">
+      <c r="F1" s="157" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="152" t="s">
+      <c r="G1" s="164" t="s">
         <v>116</v>
       </c>
-      <c r="H1" s="147" t="s">
+      <c r="H1" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="149" t="s">
+      <c r="I1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="150"/>
-      <c r="K1" s="151"/>
-      <c r="L1" s="149" t="s">
+      <c r="J1" s="155"/>
+      <c r="K1" s="163"/>
+      <c r="L1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="150"/>
-      <c r="N1" s="151"/>
-      <c r="O1" s="149" t="s">
+      <c r="M1" s="155"/>
+      <c r="N1" s="163"/>
+      <c r="O1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="150"/>
-      <c r="Q1" s="151"/>
+      <c r="P1" s="155"/>
+      <c r="Q1" s="163"/>
       <c r="S1" s="128"/>
       <c r="T1" s="128"/>
       <c r="U1" s="128"/>
       <c r="V1" s="128"/>
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
-      <c r="B2" s="163"/>
-      <c r="C2" s="157"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="160"/>
+      <c r="C2" s="152"/>
       <c r="D2" s="44"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="153"/>
-      <c r="H2" s="148"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="158"/>
+      <c r="G2" s="165"/>
+      <c r="H2" s="162"/>
       <c r="I2" s="111" t="s">
         <v>36</v>
       </c>
@@ -5349,16 +5349,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
   </mergeCells>
   <conditionalFormatting sqref="K35:K1048576 K27:K32 K1:K25">
     <cfRule type="top10" dxfId="18" priority="9" percent="1" rank="25"/>
@@ -5396,66 +5396,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="178" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="154" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="177" t="s">
+      <c r="B1" s="149" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="179" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="156" t="s">
+      <c r="D1" s="151" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="169" t="s">
+      <c r="G1" s="171" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="169" t="s">
+      <c r="H1" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="178" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="183" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="159"/>
-      <c r="B2" s="155"/>
-      <c r="C2" s="171"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="A2" s="156"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="152"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -5483,11 +5483,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="164"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="166"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="30">
@@ -5499,10 +5499,10 @@
       <c r="D3" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="179">
-        <v>0</v>
-      </c>
-      <c r="F3" s="181">
+      <c r="E3" s="180">
+        <v>0</v>
+      </c>
+      <c r="F3" s="182">
         <v>0</v>
       </c>
       <c r="G3" s="58">
@@ -5554,7 +5554,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E4" s="180"/>
+      <c r="E4" s="181"/>
       <c r="F4" s="174"/>
       <c r="G4" s="58">
         <v>35.6</v>
@@ -5608,10 +5608,10 @@
       <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="172">
+      <c r="E5" s="175">
         <v>32.700000000000003</v>
       </c>
-      <c r="F5" s="173">
+      <c r="F5" s="176">
         <v>90.1</v>
       </c>
       <c r="G5" s="58">
@@ -5664,8 +5664,8 @@
       <c r="D6" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="172"/>
-      <c r="F6" s="173"/>
+      <c r="E6" s="175"/>
+      <c r="F6" s="176"/>
       <c r="G6" s="58">
         <v>35.6</v>
       </c>
@@ -5788,10 +5788,10 @@
       <c r="D9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="172">
+      <c r="E9" s="175">
         <v>66.599999999999994</v>
       </c>
-      <c r="F9" s="173">
+      <c r="F9" s="176">
         <v>181.3</v>
       </c>
       <c r="G9" s="58">
@@ -5843,8 +5843,8 @@
       <c r="D10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="172"/>
-      <c r="F10" s="173"/>
+      <c r="E10" s="175"/>
+      <c r="F10" s="176"/>
       <c r="G10" s="58">
         <v>75.8</v>
       </c>
@@ -5894,8 +5894,8 @@
       <c r="D11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="172"/>
-      <c r="F11" s="173"/>
+      <c r="E11" s="175"/>
+      <c r="F11" s="176"/>
       <c r="G11" s="58">
         <v>89.5</v>
       </c>
@@ -5943,8 +5943,8 @@
       <c r="D12" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="172"/>
-      <c r="F12" s="173"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="176"/>
       <c r="G12" s="58">
         <v>46.1</v>
       </c>
@@ -5994,8 +5994,8 @@
       <c r="D13" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="172"/>
-      <c r="F13" s="173"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="176"/>
       <c r="G13" s="58">
         <v>73.400000000000006</v>
       </c>
@@ -6044,8 +6044,8 @@
       <c r="D14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="172"/>
-      <c r="F14" s="173"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="176"/>
       <c r="G14" s="58">
         <v>88.4</v>
       </c>
@@ -6094,8 +6094,8 @@
       <c r="D15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="173"/>
+      <c r="E15" s="175"/>
+      <c r="F15" s="176"/>
       <c r="G15" s="58">
         <v>27.5</v>
       </c>
@@ -6144,8 +6144,8 @@
       <c r="D16" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="172"/>
-      <c r="F16" s="173"/>
+      <c r="E16" s="175"/>
+      <c r="F16" s="176"/>
       <c r="G16" s="58">
         <v>94.8</v>
       </c>
@@ -6194,8 +6194,8 @@
       <c r="D17" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="172"/>
-      <c r="F17" s="173"/>
+      <c r="E17" s="175"/>
+      <c r="F17" s="176"/>
       <c r="G17" s="58">
         <v>861.6</v>
       </c>
@@ -6247,8 +6247,8 @@
       <c r="D18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="172"/>
-      <c r="F18" s="173"/>
+      <c r="E18" s="175"/>
+      <c r="F18" s="176"/>
       <c r="G18" s="58">
         <v>48.1</v>
       </c>
@@ -6297,8 +6297,8 @@
       <c r="D19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="172"/>
-      <c r="F19" s="173"/>
+      <c r="E19" s="175"/>
+      <c r="F19" s="176"/>
       <c r="G19" s="58">
         <v>41.8</v>
       </c>
@@ -6353,6 +6353,14 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="E9:E19"/>
     <mergeCell ref="F9:F19"/>
     <mergeCell ref="B1:B2"/>
@@ -6367,14 +6375,6 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:P1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
@@ -6408,10 +6408,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="193" t="s">
+      <c r="A1" s="187" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="193" t="s">
+      <c r="B1" s="187" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="188" t="s">
@@ -6423,22 +6423,22 @@
       <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="189" t="s">
+      <c r="F1" s="195" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="189"/>
-      <c r="H1" s="182" t="s">
+      <c r="G1" s="195"/>
+      <c r="H1" s="189" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="182"/>
-      <c r="J1" s="183" t="s">
+      <c r="I1" s="189"/>
+      <c r="J1" s="190" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="183"/>
+      <c r="K1" s="190"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="193"/>
-      <c r="B2" s="193"/>
+      <c r="A2" s="187"/>
+      <c r="B2" s="187"/>
       <c r="C2" s="188"/>
       <c r="D2" s="188"/>
       <c r="E2" s="188"/>
@@ -6462,16 +6462,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="184" t="s">
+      <c r="A3" s="191" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="184">
+      <c r="C3" s="191">
         <v>1550</v>
       </c>
-      <c r="D3" s="184" t="s">
+      <c r="D3" s="191" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="13">
@@ -6497,12 +6497,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="185"/>
+      <c r="A4" s="192"/>
       <c r="B4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="185"/>
-      <c r="D4" s="187"/>
+      <c r="C4" s="192"/>
+      <c r="D4" s="194"/>
       <c r="E4" s="18">
         <v>52</v>
       </c>
@@ -6526,11 +6526,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="185"/>
+      <c r="A5" s="192"/>
       <c r="B5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="185"/>
+      <c r="C5" s="192"/>
       <c r="D5" s="19" t="s">
         <v>14</v>
       </c>
@@ -6558,11 +6558,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="186"/>
+      <c r="A6" s="193"/>
       <c r="B6" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="186"/>
+      <c r="C6" s="193"/>
       <c r="D6" s="23" t="s">
         <v>15</v>
       </c>
@@ -6590,16 +6590,16 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="190" t="s">
+      <c r="A7" s="184" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="190">
+      <c r="C7" s="184">
         <v>1320</v>
       </c>
-      <c r="D7" s="190" t="s">
+      <c r="D7" s="184" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="3">
@@ -6625,12 +6625,12 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="191"/>
+      <c r="A8" s="185"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="191"/>
-      <c r="D8" s="192"/>
+      <c r="C8" s="185"/>
+      <c r="D8" s="186"/>
       <c r="E8" s="1">
         <v>100</v>
       </c>
@@ -6654,11 +6654,11 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="191"/>
+      <c r="A9" s="185"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="191"/>
+      <c r="C9" s="185"/>
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
@@ -6686,11 +6686,11 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="191"/>
+      <c r="A10" s="185"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="191"/>
+      <c r="C10" s="185"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
@@ -6718,11 +6718,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="192"/>
+      <c r="A11" s="186"/>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="192"/>
+      <c r="C11" s="186"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
@@ -6751,6 +6751,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:G1"/>
     <mergeCell ref="A7:A11"/>
     <mergeCell ref="C7:C11"/>
     <mergeCell ref="D7:D8"/>
@@ -6758,13 +6765,6 @@
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6783,10 +6783,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="193" t="s">
+      <c r="A1" s="187" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="193" t="s">
+      <c r="B1" s="187" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="188" t="s">
@@ -6798,22 +6798,22 @@
       <c r="E1" s="188" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="189" t="s">
+      <c r="F1" s="195" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="189"/>
-      <c r="H1" s="182" t="s">
+      <c r="G1" s="195"/>
+      <c r="H1" s="189" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="182"/>
-      <c r="J1" s="183" t="s">
+      <c r="I1" s="189"/>
+      <c r="J1" s="190" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="183"/>
+      <c r="K1" s="190"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="193"/>
-      <c r="B2" s="193"/>
+      <c r="A2" s="187"/>
+      <c r="B2" s="187"/>
       <c r="C2" s="188"/>
       <c r="D2" s="188"/>
       <c r="E2" s="188"/>
@@ -6837,16 +6837,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="190" t="s">
+      <c r="A3" s="184" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="190">
+      <c r="C3" s="184">
         <v>1320</v>
       </c>
-      <c r="D3" s="190" t="s">
+      <c r="D3" s="184" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="3">
@@ -6872,12 +6872,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="191"/>
+      <c r="A4" s="185"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="191"/>
-      <c r="D4" s="192"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="186"/>
       <c r="E4" s="1">
         <v>100</v>
       </c>
@@ -6901,11 +6901,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="191"/>
+      <c r="A5" s="185"/>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="191"/>
+      <c r="C5" s="185"/>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
@@ -6933,11 +6933,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="191"/>
+      <c r="A6" s="185"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="191"/>
+      <c r="C6" s="185"/>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
@@ -6965,11 +6965,11 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="192"/>
+      <c r="A7" s="186"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="192"/>
+      <c r="C7" s="186"/>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
@@ -7042,63 +7042,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="162" t="s">
+      <c r="B1" s="159" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="153" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="150" t="s">
+      <c r="E1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="152" t="s">
+      <c r="H1" s="164" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="147" t="s">
+      <c r="I1" s="161" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="149" t="s">
+      <c r="J1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="150"/>
-      <c r="L1" s="151"/>
-      <c r="M1" s="149" t="s">
+      <c r="K1" s="155"/>
+      <c r="L1" s="163"/>
+      <c r="M1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="150"/>
-      <c r="O1" s="151"/>
-      <c r="P1" s="149" t="s">
+      <c r="N1" s="155"/>
+      <c r="O1" s="163"/>
+      <c r="P1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="150"/>
-      <c r="R1" s="151"/>
+      <c r="Q1" s="155"/>
+      <c r="R1" s="163"/>
       <c r="T1" s="72"/>
       <c r="U1" s="72"/>
       <c r="V1" s="72"/>
       <c r="W1" s="128"/>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
-      <c r="B2" s="163"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="153"/>
-      <c r="I2" s="148"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="160"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="165"/>
+      <c r="I2" s="162"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
       </c>
@@ -8871,10 +8871,10 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A43" s="194" t="s">
+      <c r="A43" s="147" t="s">
         <v>182</v>
       </c>
-      <c r="B43" s="195"/>
+      <c r="B43" s="148"/>
       <c r="C43" s="38" t="s">
         <v>183</v>
       </c>
@@ -8900,28 +8900,28 @@
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A44" s="194"/>
-      <c r="B44" s="195"/>
+      <c r="A44" s="147"/>
+      <c r="B44" s="148"/>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A45" s="194"/>
-      <c r="B45" s="195"/>
+      <c r="A45" s="147"/>
+      <c r="B45" s="148"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:L1"/>
     <mergeCell ref="A43:B45"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L1:L1048576">
@@ -8960,63 +8960,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="162" t="s">
+      <c r="B1" s="159" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="151" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="149" t="s">
+      <c r="D1" s="153" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="150" t="s">
+      <c r="E1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="152" t="s">
+      <c r="H1" s="164" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="147" t="s">
+      <c r="I1" s="161" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="149" t="s">
+      <c r="J1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="150"/>
-      <c r="L1" s="151"/>
-      <c r="M1" s="149" t="s">
+      <c r="K1" s="155"/>
+      <c r="L1" s="163"/>
+      <c r="M1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="150"/>
-      <c r="O1" s="151"/>
-      <c r="P1" s="149" t="s">
+      <c r="N1" s="155"/>
+      <c r="O1" s="163"/>
+      <c r="P1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="150"/>
-      <c r="R1" s="151"/>
+      <c r="Q1" s="155"/>
+      <c r="R1" s="163"/>
       <c r="S1" s="128"/>
       <c r="T1" s="69"/>
       <c r="U1" s="69"/>
       <c r="V1" s="69"/>
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
-      <c r="B2" s="163"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="153"/>
-      <c r="I2" s="148"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="160"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="165"/>
+      <c r="I2" s="162"/>
       <c r="J2" s="111" t="s">
         <v>36</v>
       </c>
@@ -9045,8 +9045,8 @@
         <v>51</v>
       </c>
       <c r="S2" s="128"/>
-      <c r="T2" s="164"/>
-      <c r="U2" s="164"/>
+      <c r="T2" s="166"/>
+      <c r="U2" s="166"/>
       <c r="V2" s="141"/>
     </row>
     <row r="3" spans="1:22" s="30" customFormat="1" x14ac:dyDescent="0.25">
@@ -9821,65 +9821,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="151" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="165" t="s">
+      <c r="H1" s="167" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="154" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="149" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
+      <c r="A2" s="150"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="157"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="C2" s="152"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -9907,11 +9907,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="155"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="150"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -11179,11 +11179,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
@@ -11193,6 +11188,11 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <conditionalFormatting sqref="M1:M1048576">
     <cfRule type="top10" dxfId="14" priority="1" percent="1" rank="25"/>
@@ -11232,65 +11232,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="170" t="s">
+      <c r="C1" s="172" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="169" t="s">
+      <c r="H1" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="154" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="149" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
+      <c r="A2" s="150"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="171"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="C2" s="173"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -11318,11 +11318,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="155"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="150"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -12245,12 +12245,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -12259,6 +12253,12 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
@@ -12306,65 +12306,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="170" t="s">
+      <c r="C1" s="172" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="169" t="s">
+      <c r="H1" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="154" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="149" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
+      <c r="A2" s="150"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="171"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="C2" s="173"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -12392,11 +12392,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="155"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="150"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -13060,12 +13060,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -13074,6 +13068,12 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
     <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
@@ -13120,65 +13120,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="170" t="s">
+      <c r="C1" s="172" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="169" t="s">
+      <c r="H1" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="154" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="149" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
+      <c r="A2" s="150"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="171"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="C2" s="173"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -13206,11 +13206,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="155"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="150"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -13753,6 +13753,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -13761,12 +13767,6 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
@@ -13813,65 +13813,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="149" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="151" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="160" t="s">
+      <c r="G1" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="165" t="s">
+      <c r="H1" s="167" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="162" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="159" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="155"/>
+      <c r="A2" s="150"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="157"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="C2" s="152"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -13899,11 +13899,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="163"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="160"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -15143,12 +15143,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -15157,6 +15151,12 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
@@ -15213,66 +15213,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="178" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="154" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="177" t="s">
+      <c r="B1" s="149" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="179" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="156" t="s">
+      <c r="D1" s="151" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="149" t="s">
+      <c r="E1" s="153" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="150" t="s">
+      <c r="F1" s="155" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="169" t="s">
+      <c r="G1" s="171" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="169" t="s">
+      <c r="H1" s="171" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="150" t="s">
+      <c r="I1" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="J1" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="150"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="149" t="s">
+      <c r="L1" s="155"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="153" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="150"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="149" t="s">
+      <c r="O1" s="155"/>
+      <c r="P1" s="163"/>
+      <c r="Q1" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="150"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="176" t="s">
+      <c r="R1" s="155"/>
+      <c r="S1" s="163"/>
+      <c r="T1" s="178" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="159"/>
-      <c r="B2" s="155"/>
-      <c r="C2" s="171"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="168"/>
+      <c r="A2" s="156"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="152"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="156"/>
+      <c r="J2" s="170"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -15300,11 +15300,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="159"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
+      <c r="T2" s="156"/>
+      <c r="V2" s="156"/>
+      <c r="W2" s="156"/>
+      <c r="X2" s="156"/>
+      <c r="Y2" s="156"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="46">
@@ -15374,16 +15374,16 @@
       <c r="D4" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="172">
+      <c r="E4" s="175">
         <v>32.700000000000003</v>
       </c>
-      <c r="F4" s="173">
+      <c r="F4" s="176">
         <v>90.1</v>
       </c>
-      <c r="G4" s="175">
+      <c r="G4" s="177">
         <v>38.5</v>
       </c>
-      <c r="H4" s="175"/>
+      <c r="H4" s="177"/>
       <c r="I4" s="66">
         <v>18.3</v>
       </c>
@@ -15426,8 +15426,8 @@
       <c r="D5" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="172"/>
-      <c r="F5" s="173"/>
+      <c r="E5" s="175"/>
+      <c r="F5" s="176"/>
       <c r="G5" s="174">
         <v>41.2</v>
       </c>
@@ -15476,8 +15476,8 @@
       <c r="D6" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="172"/>
-      <c r="F6" s="173"/>
+      <c r="E6" s="175"/>
+      <c r="F6" s="176"/>
       <c r="G6" s="174">
         <v>24.3</v>
       </c>
@@ -15523,8 +15523,8 @@
       <c r="D7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="172"/>
-      <c r="F7" s="173"/>
+      <c r="E7" s="175"/>
+      <c r="F7" s="176"/>
       <c r="G7" s="174">
         <v>42.6</v>
       </c>
@@ -15572,8 +15572,8 @@
       <c r="D8" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="172"/>
-      <c r="F8" s="173"/>
+      <c r="E8" s="175"/>
+      <c r="F8" s="176"/>
       <c r="G8" s="174">
         <v>31.9</v>
       </c>
@@ -15619,8 +15619,8 @@
       <c r="D9" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="172"/>
-      <c r="F9" s="173"/>
+      <c r="E9" s="175"/>
+      <c r="F9" s="176"/>
       <c r="G9" s="66">
         <v>2.7</v>
       </c>
@@ -15669,8 +15669,8 @@
       <c r="D10" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="172"/>
-      <c r="F10" s="173"/>
+      <c r="E10" s="175"/>
+      <c r="F10" s="176"/>
       <c r="G10" s="58">
         <v>4.2</v>
       </c>
@@ -15719,8 +15719,8 @@
       <c r="D11" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="172"/>
-      <c r="F11" s="173"/>
+      <c r="E11" s="175"/>
+      <c r="F11" s="176"/>
       <c r="G11" s="58">
         <v>1.3</v>
       </c>
@@ -15838,10 +15838,10 @@
       <c r="D14" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="172">
+      <c r="E14" s="175">
         <v>66.599999999999994</v>
       </c>
-      <c r="F14" s="173">
+      <c r="F14" s="176">
         <v>181.3</v>
       </c>
       <c r="G14" s="174">
@@ -15889,12 +15889,12 @@
       <c r="D15" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="173"/>
-      <c r="G15" s="175">
+      <c r="E15" s="175"/>
+      <c r="F15" s="176"/>
+      <c r="G15" s="177">
         <v>68.7</v>
       </c>
-      <c r="H15" s="175"/>
+      <c r="H15" s="177"/>
       <c r="I15" s="66">
         <v>51.9</v>
       </c>
@@ -15937,12 +15937,12 @@
       <c r="D16" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="172"/>
-      <c r="F16" s="173"/>
-      <c r="G16" s="175">
+      <c r="E16" s="175"/>
+      <c r="F16" s="176"/>
+      <c r="G16" s="177">
         <v>105</v>
       </c>
-      <c r="H16" s="175"/>
+      <c r="H16" s="177"/>
       <c r="I16" s="66">
         <v>0</v>
       </c>
@@ -15985,8 +15985,8 @@
       <c r="D17" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="172"/>
-      <c r="F17" s="173"/>
+      <c r="E17" s="175"/>
+      <c r="F17" s="176"/>
       <c r="G17" s="174">
         <v>65.599999999999994</v>
       </c>
@@ -16033,8 +16033,8 @@
       <c r="D18" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="172"/>
-      <c r="F18" s="173"/>
+      <c r="E18" s="175"/>
+      <c r="F18" s="176"/>
       <c r="G18" s="58">
         <v>42.6</v>
       </c>
@@ -16083,8 +16083,8 @@
       <c r="D19" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="172"/>
-      <c r="F19" s="173"/>
+      <c r="E19" s="175"/>
+      <c r="F19" s="176"/>
       <c r="G19" s="58">
         <v>47.7</v>
       </c>
@@ -16133,8 +16133,8 @@
       <c r="D20" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="172"/>
-      <c r="F20" s="173"/>
+      <c r="E20" s="175"/>
+      <c r="F20" s="176"/>
       <c r="G20" s="58">
         <v>48.7</v>
       </c>
@@ -16290,18 +16290,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E4:E11"/>
-    <mergeCell ref="F4:F11"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="E14:E20"/>
+    <mergeCell ref="F14:F20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G14:H14"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -16313,12 +16307,18 @@
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="E14:E20"/>
-    <mergeCell ref="F14:F20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E4:E11"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">

</xml_diff>